<commit_message>
hash/sliding window method for dates updates
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,50 +545,45 @@
           <t>MVR Score</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Hire_Date_Flag</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>ABDUL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Perolis</t>
+          <t>KARIMI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>12/05/1930</t>
+          <t>09/12/1983</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>03/08/2027</t>
+          <t>11/17/2022</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>3.3</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>D01082775</t>
+          <t>39516955</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -597,7 +592,7 @@
         </is>
       </c>
       <c r="K2" s="4" t="n">
-        <v>46999</v>
+        <v>46277</v>
       </c>
       <c r="L2" t="b">
         <v>1</v>
@@ -607,51 +602,46 @@
       </c>
       <c r="U2" t="n">
         <v>0</v>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>Invalid - Manual Review</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Dennis</t>
+          <t>Abdul</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Fritch</t>
+          <t>Walizada</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>06/26/1967</t>
+          <t>09/10/1987</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>01/20/2025</t>
+          <t>12/02/2025</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1.1</v>
+        <v>0.3</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>D07630764</t>
+          <t>40727794</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -660,7 +650,7 @@
         </is>
       </c>
       <c r="K3" s="4" t="n">
-        <v>47115</v>
+        <v>47736</v>
       </c>
       <c r="L3" t="b">
         <v>1</v>
@@ -676,51 +666,46 @@
       </c>
       <c r="U3" t="n">
         <v>0</v>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>Century Corrected</t>
-        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ivan</t>
+          <t>Ahmad</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dimitrijevic</t>
+          <t>Mukhtar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>08/28/1976</t>
+          <t>07/07/1986</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>01/03/2019</t>
+          <t>05/01/2025</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>7.2</v>
+        <v>0.8</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>D09366182</t>
+          <t>40328215</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -729,7 +714,7 @@
         </is>
       </c>
       <c r="K4" s="4" t="n">
-        <v>48333</v>
+        <v>47306</v>
       </c>
       <c r="L4" t="b">
         <v>1</v>
@@ -739,51 +724,46 @@
       </c>
       <c r="U4" t="n">
         <v>0</v>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>Century Corrected</t>
-        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jared</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Henderson</t>
+          <t>ANWARI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>08/17/1978</t>
+          <t>01/01/1991</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>03/08/2028</t>
+          <t>12/17/2021</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.4</v>
+        <v>4.2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>TX</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>D02447008</t>
+          <t>41971182</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -792,90 +772,1124 @@
         </is>
       </c>
       <c r="K5" s="4" t="n">
-        <v>47021</v>
+        <v>47484</v>
       </c>
       <c r="L5" t="b">
         <v>1</v>
       </c>
-      <c r="N5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>1</v>
-      </c>
       <c r="T5" t="b">
         <v>1</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>Invalid - Manual Review</t>
-        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Jack</t>
+          <t>AHMAD</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Kelley</t>
+          <t>IRFANY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>09/19/1969</t>
+          <t>01/01/1990</t>
         </is>
       </c>
       <c r="D6" t="n">
+        <v>36</v>
+      </c>
+      <c r="E6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>03/03/2024</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>40595331</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>48580</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="T6" t="b">
+        <v>1</v>
+      </c>
+      <c r="U6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ALI</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VANNOY</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12/31/1988</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>37</v>
+      </c>
+      <c r="E7" t="n">
+        <v>11</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>06/28/2021</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Y200152009</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>47848</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="T7" t="b">
+        <v>1</v>
+      </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AMIR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TOUSSI</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>09/18/1974</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>51</v>
+      </c>
+      <c r="E8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>03/11/2025</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>37852439</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>48475</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+      <c r="T8" t="b">
+        <v>1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ARYAN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FAZLY</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>01/04/1990</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>36</v>
+      </c>
+      <c r="E9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>08/16/2020</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>39598710</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>47852</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" t="b">
+        <v>1</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bari</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Safi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>06/01/1992</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>33</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>12/16/2025</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>45505317</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>47270</v>
+      </c>
+      <c r="L10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FRAIDOON</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FAZEL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>11/30/1983</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>42</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>10/28/2021</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>39389242</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>48548</v>
+      </c>
+      <c r="L11" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" t="b">
+        <v>1</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Habibullah</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Nejat</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>02/16/1995</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>31</v>
+      </c>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>12/29/2025</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>47447879</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>48260</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="T12" t="b">
+        <v>1</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Hashmatullah</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Noori</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>04/11/1992</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>33</v>
+      </c>
+      <c r="E13" t="n">
+        <v>11</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>01/01/2019</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>41058085</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>47949</v>
+      </c>
+      <c r="L13" t="b">
+        <v>1</v>
+      </c>
+      <c r="T13" t="b">
+        <v>1</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hosseinali</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Jokar</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>05/05/1969</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>56</v>
       </c>
-      <c r="E6" t="n">
-        <v>12</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>09/11/2025</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>35771642</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>48704</v>
+      </c>
+      <c r="L14" t="b">
+        <v>1</v>
+      </c>
+      <c r="T14" t="b">
+        <v>1</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>JAMSHID</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ANWARI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>07/08/1985</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>04/01/2021</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>38622685</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>48768</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
+      </c>
+      <c r="T15" t="b">
+        <v>1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rahimi</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>01/01/1985</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>41</v>
+      </c>
+      <c r="E16" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>07/02/2025</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>39300242</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>47849</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="T16" t="b">
+        <v>1</v>
+      </c>
+      <c r="U16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MOHAMMAD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>AZIZI</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>06/22/1986</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>39</v>
+      </c>
+      <c r="E17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>02/16/2023</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>41000925</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>48752</v>
+      </c>
+      <c r="L17" t="b">
+        <v>1</v>
+      </c>
+      <c r="T17" t="b">
+        <v>1</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MUSTAF</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HIDARY</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>07/04/1984</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>41</v>
+      </c>
+      <c r="E18" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>09/28/2023</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>X200297004</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>46572</v>
+      </c>
+      <c r="L18" t="b">
+        <v>1</v>
+      </c>
+      <c r="T18" t="b">
+        <v>1</v>
+      </c>
+      <c r="U18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Omidullah</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ibrahimi</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>07/22/1993</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>32</v>
+      </c>
+      <c r="E19" t="n">
+        <v>8</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>01/14/2026</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>5270462642</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>46225</v>
+      </c>
+      <c r="L19" t="b">
+        <v>1</v>
+      </c>
+      <c r="T19" t="b">
+        <v>1</v>
+      </c>
+      <c r="U19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>SAKHIKHAN</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>REZAYEE</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>01/01/1990</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>36</v>
+      </c>
+      <c r="E20" t="n">
+        <v>14</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>39225451</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>47484</v>
+      </c>
+      <c r="L20" t="b">
+        <v>1</v>
+      </c>
+      <c r="T20" t="b">
+        <v>1</v>
+      </c>
+      <c r="U20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>SAYED</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HASHEMI</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>01/01/1989</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>37</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>02/25/2025</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>41514811</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>47484</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
+      <c r="T21" t="b">
+        <v>1</v>
+      </c>
+      <c r="U21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tariq</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Zia</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>11/28/1982</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>43</v>
+      </c>
+      <c r="E22" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>01/06/2026</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="G22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>42951664</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>47085</v>
+      </c>
+      <c r="L22" t="b">
+        <v>1</v>
+      </c>
+      <c r="N22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>1</v>
+      </c>
+      <c r="T22" t="b">
+        <v>1</v>
+      </c>
+      <c r="U22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wahid</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rahimi</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>07/20/1988</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>37</v>
+      </c>
+      <c r="E23" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>12/30/2025</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>44562640</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>48049</v>
+      </c>
+      <c r="L23" t="b">
+        <v>1</v>
+      </c>
+      <c r="T23" t="b">
+        <v>1</v>
+      </c>
+      <c r="U23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PEDRAM</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>FREEMAN</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>02/09/1994</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>32</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>01/19/2026</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
         <v>0.1</v>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>D00356824</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>46649</v>
-      </c>
-      <c r="L6" t="b">
-        <v>1</v>
-      </c>
-      <c r="T6" t="b">
-        <v>1</v>
-      </c>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>Century Corrected</t>
-        </is>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>37981621</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>48619</v>
+      </c>
+      <c r="L24" t="b">
+        <v>1</v>
+      </c>
+      <c r="T24" t="b">
+        <v>1</v>
+      </c>
+      <c r="U24" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>